<commit_message>
Sprint Backlog S4: cierre de tareas HU-084/086/094/100/103/160
Marca Terminada las tareas de Emilio y deja las historias En revision
(pruebas/documentacion de terceros pendientes). Incluye las observaciones
de cada tarea. HU-103: las de API quedan En revision por indicacion.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S4.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S4.xlsx
@@ -197,7 +197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -254,6 +254,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1166,6 +1169,8 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5" ht="27.75" customHeight="1" s="19">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -1603,7 +1608,7 @@
       </c>
       <c r="P10" s="17" t="inlineStr">
         <is>
-          <t>Construida por Emilio Fuentes (11-09-2026) siguiendo PATRONES/ASP: BD SEL/INS/UPD/DEL_CHECKLIST_PLANTILLA (patron dinamico, FNC_PAIS_HORA, INS_EXCEPCION, codigo unico por cliente, baja logica) + estructura Version/Seccion/Item/Validacion (BD/192) + lookups (BD/189,191,194). Web: ChecklistPlantillas/ChecklistPlantilla/ChecklistPlantillaVista con Model+Controllers; editor inline de secciones y campos; previsualizacion de solo lectura al clic. Datos reales: SOP-09-R24 con 25 secciones y 208 campos (BD/193). Seguridad por cliente + Token + Menu_Funcion. Compila exitcode=0 y SP probados en transaccion revertida. PENDIENTE (otra persona): pruebas por criterio, documentacion y consumo movil.</t>
+          <t>Construida por Emilio Fuentes (11-09-2026) siguiendo PATRONES/ASP: BD SEL/INS/UPD/DEL_CHECKLIST_PLANTILLA (patron dinamico, FNC_PAIS_HORA, INS_EXCEPCION, codigo unico por cliente, baja logica) + estructura Version/Seccion/Item/Validacion (BD/192) + lookups (BD/189,191,194). Web: ChecklistPlantillas/ChecklistPlantilla/ChecklistPlantillaVista con Model+Controllers; editor inline de secciones y campos; previsualizacion de solo lectura al clic. Datos reales: SOP-09-R24 con 25 secciones y 208 campos (BD/193). Seguridad por cliente + Token + Menu_Funcion. Compila exitcode=0 y SP probados en transaccion revertida. PENDIENTE (otra persona): pruebas por criterio, documentacion y consumo movil. || AJUSTE 21-09-2026 (Emilio Fuentes): se unifico el termino en la interfaz a "Pauta de inspeccion" y se quito "checklist" del texto visible (titulo de la ficha, seccion "Campos de la pauta", ayudas y mensajes de exito). Los nombres tecnicos internos (tablas Checklist_*, SP, clases, archivos) NO cambian; es solo lenguaje de cara al usuario para no mezclar "pauta" y "checklist".</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1815,7 @@
       </c>
       <c r="N13" s="13" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="O13" s="14" t="inlineStr">
@@ -1818,7 +1823,11 @@
           <t>Emilio Fuentes</t>
         </is>
       </c>
-      <c r="P13" s="14" t="n"/>
+      <c r="P13" s="14" t="inlineStr">
+        <is>
+          <t>BD (SPs+índices+datos), Web PlanVersion.aspx y Seguridad terminadas (Emilio). Pendiente: pruebas (T-4119) y documentación (T-4120) de Bryan.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="96.59999999999999" customHeight="1" s="19">
       <c r="A14" s="11" t="inlineStr">
@@ -2027,7 +2036,7 @@
       </c>
       <c r="N16" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="O16" s="12" t="inlineStr">
@@ -2035,7 +2044,11 @@
           <t>Emilio Fuentes</t>
         </is>
       </c>
-      <c r="P16" s="12" t="n"/>
+      <c r="P16" s="12" t="inlineStr">
+        <is>
+          <t>Backend terminado (Emilio): BD (SEL/INS/datos+índices), API GET/POST /dictado-voz/sync, middleware de suscripción 402 y seguridad. Pendiente: móvil Flutter (T-4160/61/62) y pruebas/doc/validación de Catalina (T-4164/65/66).</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="96.59999999999999" customHeight="1" s="19">
       <c r="A17" s="13" t="inlineStr">
@@ -2098,7 +2111,7 @@
       </c>
       <c r="N17" s="13" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="O17" s="14" t="inlineStr">
@@ -2106,7 +2119,11 @@
           <t>Emilio Fuentes</t>
         </is>
       </c>
-      <c r="P17" s="14" t="n"/>
+      <c r="P17" s="14" t="inlineStr">
+        <is>
+          <t>BD (SP reprogramar+SEL+datos), Web PlanOcurrenciaReprogramar.aspx y Seguridad terminadas (Emilio). Pendiente pruebas/documentación.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="55.2" customHeight="1" s="19">
       <c r="A18" s="11" t="inlineStr">
@@ -2240,7 +2257,7 @@
       </c>
       <c r="N19" s="13" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="O19" s="14" t="inlineStr">
@@ -2248,7 +2265,11 @@
           <t>Emilio Fuentes</t>
         </is>
       </c>
-      <c r="P19" s="14" t="n"/>
+      <c r="P19" s="26" t="inlineStr">
+        <is>
+          <t>Construida por Emilio Fuentes (21-09-2026): BD PUBLICAR_CHECKLIST_VERSION (proceso en transaccion, retira publicada anterior, rechaza sin items, sella quien/cuando) + SEL_CHECKLIST_VERSION (BD/195,196). Web ChecklistVersion.aspx abierta desde el listado de Pautas. Seguridad por cliente + Token. Compila exitcode=0; proceso verificado en transaccion revertida. PENDIENTE (Bryan): pruebas y documentacion.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="69" customHeight="1" s="19">
       <c r="A20" s="11" t="inlineStr">
@@ -2311,7 +2332,7 @@
       </c>
       <c r="N20" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="O20" s="12" t="inlineStr">
@@ -2319,7 +2340,11 @@
           <t>Emilio Fuentes</t>
         </is>
       </c>
-      <c r="P20" s="12" t="n"/>
+      <c r="P20" s="17" t="inlineStr">
+        <is>
+          <t>Construida por Emilio Fuentes (22-09-2026): BD SEL/INS/UPD_CHECKLIST_PROGRAMACION (resuelve version publicada, exige activo O area, FNC_PAIS_HORA, patron dinamico) + datos de prueba (BD/197, 198). Web ChecklistProgramacions/ChecklistProgramacion con Model+Controller; combos por SEL_. Seguridad por cliente + Token. Compila exitcode=0; CA3 verificado en transaccion revertida. NOTA: para programar una pauta debe estar PUBLICADA (HU-093). PENDIENTE (Catalina): pruebas y documentacion.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="55.2" customHeight="1" s="19">
       <c r="A21" s="13" t="inlineStr">
@@ -2524,7 +2549,7 @@
       </c>
       <c r="N23" s="13" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="O23" s="14" t="inlineStr">
@@ -2532,7 +2557,11 @@
           <t>Emilio Fuentes</t>
         </is>
       </c>
-      <c r="P23" s="14" t="n"/>
+      <c r="P23" s="14" t="inlineStr">
+        <is>
+          <t>BD (SEL+datos+modelo) y Seguridad terminadas (Emilio). API (GET/POST sync + middleware) en revisión, para otro momento. Móvil y pruebas/doc según reparto.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="69" customHeight="1" s="19">
       <c r="A24" s="11" t="inlineStr">
@@ -2879,7 +2908,7 @@
       </c>
       <c r="N28" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="O28" s="12" t="inlineStr">
@@ -2887,7 +2916,11 @@
           <t>Emilio Fuentes</t>
         </is>
       </c>
-      <c r="P28" s="12" t="n"/>
+      <c r="P28" s="12" t="inlineStr">
+        <is>
+          <t>BD (modelo+SEL/INS/UPD/DEL+datos), Web (listado+ficha+menú) y Seguridad terminadas (Emilio). Pendiente pruebas/documentación.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="55.2" customHeight="1" s="19">
       <c r="A29" s="13" t="inlineStr">
@@ -3070,8 +3103,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="27.75" customHeight="1" s="19">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -6812,11 +6843,15 @@
       </c>
       <c r="H92" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I92" s="11" t="n"/>
-      <c r="J92" s="12" t="n"/>
+      <c r="J92" s="12" t="inlineStr">
+        <is>
+          <t>Índices únicos verificados: UX_PMA_CLIENTE_CODIGO (código por cliente) y UX_PMV_PLAN_NUMERO (número por plan). Modelo Plan_Mantenimiento_Version OK.</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="27.6" customHeight="1" s="19">
       <c r="A93" s="11" t="inlineStr">
@@ -6854,11 +6889,15 @@
       </c>
       <c r="H93" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I93" s="11" t="n"/>
-      <c r="J93" s="12" t="n"/>
+      <c r="J93" s="12" t="inlineStr">
+        <is>
+          <t>Endurecido en BD/199: SET XACT_ABORT ON en UPD_PLAN_MANTENIMIENTO_VERSION_PUBLICAR y UPD_PLAN_VERSION_PUBLICAR. Publica dentro de transacción con TRY/CATCH; cualquier error revierte todo.</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="27.6" customHeight="1" s="19">
       <c r="A94" s="11" t="inlineStr">
@@ -6896,11 +6935,15 @@
       </c>
       <c r="H94" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I94" s="11" t="n"/>
-      <c r="J94" s="12" t="n"/>
+      <c r="J94" s="12" t="inlineStr">
+        <is>
+          <t>Reglas en el SP (existe, es borrador, exige hitos y equipos, decide la carrera en el UPDATE del borrador). Verificado: rechaza sin hitos (msg 3) y de otro cliente (msg 1).</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="27.6" customHeight="1" s="19">
       <c r="A95" s="11" t="inlineStr">
@@ -6938,11 +6981,15 @@
       </c>
       <c r="H95" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I95" s="11" t="n"/>
-      <c r="J95" s="12" t="n"/>
+      <c r="J95" s="12" t="inlineStr">
+        <is>
+          <t>SEL_PLAN_VERSION devuelve el historial + código/nombre del plan, conteos (hitos/activos/ocurrencias) y usuarios. Lo consume PlanVersionController.GetVersiones.</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="55.2" customHeight="1" s="19">
       <c r="A96" s="11" t="inlineStr">
@@ -6980,11 +7027,15 @@
       </c>
       <c r="H96" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I96" s="11" t="n"/>
-      <c r="J96" s="12" t="n"/>
+      <c r="J96" s="12" t="inlineStr">
+        <is>
+          <t>Datos de prueba presentes: planes PMA-* con versiones en BORRADOR/PUBLICADO/RETIRADO. Publicación probada en transacción revertida (pmv 2 → PUBLICADO, sella usuario y observación).</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="41.4" customHeight="1" s="19">
       <c r="A97" s="11" t="inlineStr">
@@ -7022,11 +7073,15 @@
       </c>
       <c r="H97" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I97" s="11" t="n"/>
-      <c r="J97" s="12" t="n"/>
+      <c r="J97" s="12" t="inlineStr">
+        <is>
+          <t>Web PlanVersion.aspx creada en View/Mantenimiento/Planes/: historial de versiones + publicar el borrador, mostrando quién publicó y cuándo. Modelo PlanVersion + PlanVersionController. Compila exitcode 0.</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="41.4" customHeight="1" s="19">
       <c r="A98" s="11" t="inlineStr">
@@ -7064,11 +7119,15 @@
       </c>
       <c r="H98" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I98" s="11" t="n"/>
-      <c r="J98" s="12" t="n"/>
+      <c r="J98" s="12" t="inlineStr">
+        <is>
+          <t>Seguridad server-side: Token.Puede('CREAR EDITAR PLANES MANTENIMIENTO') revalidado en btnPublicar_Click (no se esconde el botón). Página registrada en Menus con permiso VER PLANES MANTENIMIENTO (BD/200). Filtro por cliente en el SP.</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="41.4" customHeight="1" s="19">
       <c r="A99" s="11" t="inlineStr">
@@ -8282,11 +8341,15 @@
       </c>
       <c r="H127" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I127" s="11" t="n"/>
-      <c r="J127" s="12" t="n"/>
+      <c r="J127" s="12" t="inlineStr">
+        <is>
+          <t>Modelo verificado: Dictado_Voz existe. Su clave natural es el UUID del teléfono (no un código por cliente); el índice único UX_DVO_UUID hace idempotente la recepción. IX_DVO_CLIENTE_FECHA presente.</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="41.4" customHeight="1" s="19">
       <c r="A128" s="11" t="inlineStr">
@@ -8324,11 +8387,15 @@
       </c>
       <c r="H128" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I128" s="11" t="n"/>
-      <c r="J128" s="12" t="n"/>
+      <c r="J128" s="12" t="inlineStr">
+        <is>
+          <t>BD/201: API_SEL_DICTADO_VOZ (descarga acotada al usuario y su cliente, incremental por @DESDE). Probado: devuelve el dictado del usuario demo.</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="41.4" customHeight="1" s="19">
       <c r="A129" s="11" t="inlineStr">
@@ -8366,11 +8433,15 @@
       </c>
       <c r="H129" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I129" s="11" t="n"/>
-      <c r="J129" s="12" t="n"/>
+      <c r="J129" s="12" t="inlineStr">
+        <is>
+          <t>API_INS_DICTADO_VOZ verificado: idempotente por UUID (si el UUID ya existe devuelve el mismo id, no inserta un segundo). El audio no se guarda; nace en PROCESADO.</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="41.4" customHeight="1" s="19">
       <c r="A130" s="11" t="inlineStr">
@@ -8408,11 +8479,15 @@
       </c>
       <c r="H130" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I130" s="11" t="n"/>
-      <c r="J130" s="12" t="n"/>
+      <c r="J130" s="12" t="inlineStr">
+        <is>
+          <t>BD/201: datos de prueba (2 dictados del usuario del cliente 1 con UUID fijos, reaplicables). Cliente 1 con dictados para ejercitar los CA.</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="27.6" customHeight="1" s="19">
       <c r="A131" s="11" t="inlineStr">
@@ -8450,11 +8525,15 @@
       </c>
       <c r="H131" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I131" s="11" t="n"/>
-      <c r="J131" s="12" t="n"/>
+      <c r="J131" s="12" t="inlineStr">
+        <is>
+          <t>API GET /dictado-voz/sync — descarga para el dispositivo, identidad del token (usuario+cliente), incremental por ?desde. Compila (MSBuild exit 0).</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="41.4" customHeight="1" s="19">
       <c r="A132" s="11" t="inlineStr">
@@ -8492,11 +8571,15 @@
       </c>
       <c r="H132" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I132" s="11" t="n"/>
-      <c r="J132" s="12" t="n"/>
+      <c r="J132" s="12" t="inlineStr">
+        <is>
+          <t>API POST /dictado-voz/sync — subida por lotes, idempotente por uuid (reenvío devuelve el mismo id). Identidad del token, nunca del cuerpo.</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="41.4" customHeight="1" s="19">
       <c r="A133" s="11" t="inlineStr">
@@ -8534,11 +8617,15 @@
       </c>
       <c r="H133" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I133" s="11" t="n"/>
-      <c r="J133" s="12" t="n"/>
+      <c r="J133" s="12" t="inlineStr">
+        <is>
+          <t>Middleware SuscripcionVigenteHandler (registrado en WebApiConfig): valida la KEY del cliente (X-Cliente-Key) contra FNC_SUSCRIPCION_VIGENTE (vía API_SEL_SUSCRIPCION_VIGENTE) y responde 402 si no puede operar. Sin la KEY no corta (no rompe a nadie). Probado: hash real → PUEDE_OPERAR=1; hash inexistente → vacío → 402.</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="41.4" customHeight="1" s="19">
       <c r="A134" s="11" t="inlineStr">
@@ -8702,11 +8789,15 @@
       </c>
       <c r="H137" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I137" s="11" t="n"/>
-      <c r="J137" s="12" t="n"/>
+      <c r="J137" s="12" t="inlineStr">
+        <is>
+          <t>Seguridad server-side: identidad del token (ExigirUsuario) + acotado por cliente (ExigirCliente); el dictado no es un recurso con permiso propio (es ambiente a cualquier campo que el usuario ya edita), así que no se esconde nada por CSS y la suscripción la corta el 402 del middleware.</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="27.6" customHeight="1" s="19">
       <c r="A138" s="11" t="inlineStr">
@@ -8870,11 +8961,15 @@
       </c>
       <c r="H141" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I141" s="11" t="n"/>
-      <c r="J141" s="12" t="n"/>
+      <c r="J141" s="12" t="inlineStr">
+        <is>
+          <t>Modelo verificado: Plan_Mantenimiento_Ocurrencia con índices únicos UX_PMO_UUID, UX_PMO_HITO_ACTIVO_FECHA y UX_PMO_PROGRAMACION_ACTIVO_FECHA (impiden dos ocurrencias del mismo hito/equipo en la misma fecha). No hay 'código'; la clave es hito+activo+fecha.</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="27.6" customHeight="1" s="19">
       <c r="A142" s="11" t="inlineStr">
@@ -8912,11 +9007,15 @@
       </c>
       <c r="H142" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I142" s="11" t="n"/>
-      <c r="J142" s="12" t="n"/>
+      <c r="J142" s="12" t="inlineStr">
+        <is>
+          <t>BD/202: PLAN_OCURRENCIA_REPROGRAMAR con SET XACT_ABORT ON; todo el proceso (retirar la vieja a REPROGRAMADA + crear la nueva PENDIENTE ligada por origen) en una transacción con TRY/CATCH.</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="27.6" customHeight="1" s="19">
       <c r="A143" s="11" t="inlineStr">
@@ -8954,11 +9053,15 @@
       </c>
       <c r="H143" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I143" s="11" t="n"/>
-      <c r="J143" s="12" t="n"/>
+      <c r="J143" s="12" t="inlineStr">
+        <is>
+          <t>Reglas en el SP: solo reprograma PENDIENTE/DISPONIBLE, motivo obligatorio, fecha distinta, sin colisión de fecha, y decide la carrera en el UPDATE. Verificado: rechazos 1 (no existe/cliente ajeno), 2 (estado), 3 (motivo).</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="27.6" customHeight="1" s="19">
       <c r="A144" s="11" t="inlineStr">
@@ -8996,11 +9099,15 @@
       </c>
       <c r="H144" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I144" s="11" t="n"/>
-      <c r="J144" s="12" t="n"/>
+      <c r="J144" s="12" t="inlineStr">
+        <is>
+          <t>BD/202: SEL_PLAN_OCURRENCIA_REPROGRAMAR devuelve la ficha (activo/hito/plan, estado, fecha programada/original) y el resultado (a qué fecha se movió, la nueva ocurrencia, quién y cuándo).</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="41.4" customHeight="1" s="19">
       <c r="A145" s="11" t="inlineStr">
@@ -9038,11 +9145,15 @@
       </c>
       <c r="H145" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I145" s="11" t="n"/>
-      <c r="J145" s="12" t="n"/>
+      <c r="J145" s="12" t="inlineStr">
+        <is>
+          <t>BD/202: datos de prueba (una ocurrencia reprogramada, siembra idempotente). Además ya existían decenas de ocurrencias PENDIENTE del plan de hornos para ejercitar los CA.</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="27.6" customHeight="1" s="19">
       <c r="A146" s="11" t="inlineStr">
@@ -9080,11 +9191,15 @@
       </c>
       <c r="H146" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I146" s="11" t="n"/>
-      <c r="J146" s="12" t="n"/>
+      <c r="J146" s="12" t="inlineStr">
+        <is>
+          <t>Web PlanOcurrenciaReprogramar.aspx (View/Mantenimiento/Planes/): muestra la ocurrencia, permite mover a nueva fecha con motivo obligatorio, y muestra el resultado (movida a X por quién). Modelo PlanOcurrencia + PlanOcurrenciaController. Compila exitcode 0.</t>
+        </is>
+      </c>
     </row>
     <row r="147" ht="27.6" customHeight="1" s="19">
       <c r="A147" s="11" t="inlineStr">
@@ -9122,11 +9237,15 @@
       </c>
       <c r="H147" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I147" s="11" t="n"/>
-      <c r="J147" s="12" t="n"/>
+      <c r="J147" s="12" t="inlineStr">
+        <is>
+          <t>Seguridad server-side: Token.Puede('CREAR EDITAR PLANES MANTENIMIENTO') revalidado en btnReprogramar_Click (no se esconde el botón). Página registrada en Menus con permiso VER PLANES MANTENIMIENTO (BD/203). Filtro por cliente en el SP.</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="27.6" customHeight="1" s="19">
       <c r="A148" s="11" t="inlineStr">
@@ -9584,11 +9703,15 @@
       </c>
       <c r="H158" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I158" s="11" t="n"/>
-      <c r="J158" s="12" t="n"/>
+      <c r="J158" s="17" t="inlineStr">
+        <is>
+          <t>Revisado Checklist_Plantilla_Version; confirmado el unico UX_CPV_PLANTILLA_NUMERO. BD/195.</t>
+        </is>
+      </c>
     </row>
     <row r="159" ht="41.4" customHeight="1" s="19">
       <c r="A159" s="11" t="inlineStr">
@@ -9626,11 +9749,15 @@
       </c>
       <c r="H159" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I159" s="11" t="n"/>
-      <c r="J159" s="12" t="n"/>
+      <c r="J159" s="17" t="inlineStr">
+        <is>
+          <t>PUBLICAR_CHECKLIST_VERSION: proceso en transaccion con SET XACT_ABORT ON; FNC_PAIS_HORA + INS_EXCEPCION. BD/195.</t>
+        </is>
+      </c>
     </row>
     <row r="160" ht="27.6" customHeight="1" s="19">
       <c r="A160" s="11" t="inlineStr">
@@ -9668,11 +9795,15 @@
       </c>
       <c r="H160" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I160" s="11" t="n"/>
-      <c r="J160" s="12" t="n"/>
+      <c r="J160" s="17" t="inlineStr">
+        <is>
+          <t>Reglas en el SP: retira la publicada anterior (CA1), registra quien/cuando, rechaza publicar sin items (CA2). BD/195.</t>
+        </is>
+      </c>
     </row>
     <row r="161" ht="27.6" customHeight="1" s="19">
       <c r="A161" s="11" t="inlineStr">
@@ -9710,11 +9841,15 @@
       </c>
       <c r="H161" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I161" s="11" t="n"/>
-      <c r="J161" s="12" t="n"/>
+      <c r="J161" s="17" t="inlineStr">
+        <is>
+          <t>SEL_CHECKLIST_VERSION: historial de versiones por pauta, filtrado por cliente. BD/195.</t>
+        </is>
+      </c>
     </row>
     <row r="162" ht="27.6" customHeight="1" s="19">
       <c r="A162" s="11" t="inlineStr">
@@ -9752,11 +9887,15 @@
       </c>
       <c r="H162" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I162" s="11" t="n"/>
-      <c r="J162" s="12" t="n"/>
+      <c r="J162" s="17" t="inlineStr">
+        <is>
+          <t>Datos de prueba: borrador de SOP-09-R24 (208 items) publicable; rechazos verificados en transaccion revertida. BD/195.</t>
+        </is>
+      </c>
     </row>
     <row r="163" ht="41.4" customHeight="1" s="19">
       <c r="A163" s="11" t="inlineStr">
@@ -9794,11 +9933,15 @@
       </c>
       <c r="H163" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I163" s="11" t="n"/>
-      <c r="J163" s="12" t="n"/>
+      <c r="J163" s="17" t="inlineStr">
+        <is>
+          <t>ChecklistVersion.aspx: historial + publicar borrador, abierta desde el listado de Pautas. Model+Controller ChecklistVersion.</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="55.2" customHeight="1" s="19">
       <c r="A164" s="11" t="inlineStr">
@@ -9836,11 +9979,15 @@
       </c>
       <c r="H164" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I164" s="11" t="n"/>
-      <c r="J164" s="12" t="n"/>
+      <c r="J164" s="17" t="inlineStr">
+        <is>
+          <t>Seguridad: VER PAUTAS para abrir (Menus BD/196) + Token.Puede("CREAR EDITAR PAUTAS") para publicar; SP filtra por cliente.</t>
+        </is>
+      </c>
     </row>
     <row r="165" ht="27.6" customHeight="1" s="19">
       <c r="A165" s="11" t="inlineStr">
@@ -9962,11 +10109,15 @@
       </c>
       <c r="H167" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I167" s="11" t="n"/>
-      <c r="J167" s="12" t="n"/>
+      <c r="J167" s="17" t="inlineStr">
+        <is>
+          <t>Revisado Checklist_Programacion (FK a version, programacion, activo, area, grupo, responsable). PK cpr_id; no hay unico natural (una version se programa en varios objetivos). BD/197.</t>
+        </is>
+      </c>
     </row>
     <row r="168" ht="55.2" customHeight="1" s="19">
       <c r="A168" s="11" t="inlineStr">
@@ -10004,11 +10155,15 @@
       </c>
       <c r="H168" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I168" s="11" t="n"/>
-      <c r="J168" s="12" t="n"/>
+      <c r="J168" s="17" t="inlineStr">
+        <is>
+          <t>INS_CHECKLIST_PROGRAMACION: alta en transaccion; resuelve la version PUBLICADA de la pauta; exige activo O area (CA3); valida objetivo del cliente; FNC_PAIS_HORA + INS_EXCEPCION. BD/197.</t>
+        </is>
+      </c>
     </row>
     <row r="169" ht="41.4" customHeight="1" s="19">
       <c r="A169" s="11" t="inlineStr">
@@ -10046,11 +10201,15 @@
       </c>
       <c r="H169" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I169" s="11" t="n"/>
-      <c r="J169" s="12" t="n"/>
+      <c r="J169" s="17" t="inlineStr">
+        <is>
+          <t>SEL_CHECKLIST_PROGRAMACION: patron dinamico @SELECT/@FROM/@WHERE con nombres de pauta/recurrencia/objetivo/responsable; un solo SP grilla+ficha. BD/197.</t>
+        </is>
+      </c>
     </row>
     <row r="170" ht="41.4" customHeight="1" s="19">
       <c r="A170" s="11" t="inlineStr">
@@ -10088,11 +10247,15 @@
       </c>
       <c r="H170" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I170" s="11" t="n"/>
-      <c r="J170" s="12" t="n"/>
+      <c r="J170" s="17" t="inlineStr">
+        <is>
+          <t>UPD_CHECKLIST_PROGRAMACION: @ID/@USUARIO obligatorios, ISNULL en lo opcional, conserva la regla activo/area; puede cambiar pauta (re-resuelve version publicada). BD/197.</t>
+        </is>
+      </c>
     </row>
     <row r="171" ht="27.6" customHeight="1" s="19">
       <c r="A171" s="11" t="inlineStr">
@@ -10130,11 +10293,15 @@
       </c>
       <c r="H171" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I171" s="11" t="n"/>
-      <c r="J171" s="12" t="n"/>
+      <c r="J171" s="17" t="inlineStr">
+        <is>
+          <t>Datos de prueba: se publico SOP-09-R24 y se creo la programacion "Ronda diaria - Revolvedora 1"; CA3 (sin objetivo) verificado en transaccion revertida. BD/197.</t>
+        </is>
+      </c>
     </row>
     <row r="172" ht="41.4" customHeight="1" s="19">
       <c r="A172" s="11" t="inlineStr">
@@ -10172,11 +10339,15 @@
       </c>
       <c r="H172" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I172" s="11" t="n"/>
-      <c r="J172" s="12" t="n"/>
+      <c r="J172" s="17" t="inlineStr">
+        <is>
+          <t>ChecklistProgramacion.aspx (RadWindow, sigma-modal-* seccionada: Identificacion, Objetivo, Asignacion); combos Pauta(publicadas)/Recurrencia/Activo/Area/Grupo/Responsable por SEL_; validaciones + wuc:Auditoria.</t>
+        </is>
+      </c>
     </row>
     <row r="173" ht="55.2" customHeight="1" s="19">
       <c r="A173" s="11" t="inlineStr">
@@ -10214,11 +10385,15 @@
       </c>
       <c r="H173" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I173" s="11" t="n"/>
-      <c r="J173" s="12" t="n"/>
+      <c r="J173" s="17" t="inlineStr">
+        <is>
+          <t>ChecklistProgramacions.aspx: grilla + wucFiltro (habilitado) + Nuevo/Dar de baja; columna Objetivo (activo o area) y pauta con su version. Model+Controller ChecklistProgramacion.</t>
+        </is>
+      </c>
     </row>
     <row r="174" ht="27.6" customHeight="1" s="19">
       <c r="A174" s="11" t="inlineStr">
@@ -10256,11 +10431,15 @@
       </c>
       <c r="H174" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I174" s="11" t="n"/>
-      <c r="J174" s="12" t="n"/>
+      <c r="J174" s="17" t="inlineStr">
+        <is>
+          <t>Seguridad: VER PAUTAS para abrir (Menus BD/198) + Token.Puede("CREAR EDITAR PAUTAS") en la ficha; SEL/INS/UPD filtran por cliente.</t>
+        </is>
+      </c>
     </row>
     <row r="175" ht="27.6" customHeight="1" s="19">
       <c r="A175" s="11" t="inlineStr">
@@ -11306,11 +11485,15 @@
       </c>
       <c r="H199" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I199" s="11" t="n"/>
-      <c r="J199" s="12" t="n"/>
+      <c r="J199" s="12" t="inlineStr">
+        <is>
+          <t>Modelo verificado: Tarea_Ejecucion con UX_TEJ_UUID (idempotencia por uuid). Sin columna de cliente: el cliente sale por tej_tarea_ocurrencia -&gt; Tarea_Ocurrencia. No hay 'código por cliente'.</t>
+        </is>
+      </c>
     </row>
     <row r="200" ht="41.4" customHeight="1" s="19">
       <c r="A200" s="11" t="inlineStr">
@@ -11348,11 +11531,15 @@
       </c>
       <c r="H200" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I200" s="11" t="n"/>
-      <c r="J200" s="12" t="n"/>
+      <c r="J200" s="12" t="inlineStr">
+        <is>
+          <t>BD/204: SEL_TAREA_EJECUCION (descarga acotada al usuario, su cliente y las plantas donde está asignado, incremental por @DESDE). Probado: usuario 7 baja su ejecución; usuario sin planta no baja nada.</t>
+        </is>
+      </c>
     </row>
     <row r="201" ht="55.2" customHeight="1" s="19">
       <c r="A201" s="11" t="inlineStr">
@@ -11390,11 +11577,15 @@
       </c>
       <c r="H201" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I201" s="11" t="n"/>
-      <c r="J201" s="12" t="n"/>
+      <c r="J201" s="12" t="inlineStr">
+        <is>
+          <t>Verificado: API_UPS_TAREA_EJECUCION es idempotente por uuid (busca por uuid antes de mirar el estado; el reenvío de un cierre ya grabado no duplica ni da error falso).</t>
+        </is>
+      </c>
     </row>
     <row r="202" ht="41.4" customHeight="1" s="19">
       <c r="A202" s="11" t="inlineStr">
@@ -11432,11 +11623,15 @@
       </c>
       <c r="H202" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I202" s="11" t="n"/>
-      <c r="J202" s="12" t="n"/>
+      <c r="J202" s="12" t="inlineStr">
+        <is>
+          <t>BD/204: datos de prueba (una ejecución cerrada del usuario 7 sobre la ocurrencia 1, uuid fijo, idempotente). Ya existían 8 ejecuciones más.</t>
+        </is>
+      </c>
     </row>
     <row r="203" ht="41.4" customHeight="1" s="19">
       <c r="A203" s="11" t="inlineStr">
@@ -11474,11 +11669,15 @@
       </c>
       <c r="H203" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="I203" s="11" t="n"/>
-      <c r="J203" s="12" t="n"/>
+      <c r="J203" s="12" t="inlineStr">
+        <is>
+          <t>Pendiente (por indicación, para otro momento). El middleware de suscripción global (SuscripcionVigenteHandler, HU-160) ya aplica a estos endpoints cuando se construyan.</t>
+        </is>
+      </c>
     </row>
     <row r="204" ht="41.4" customHeight="1" s="19">
       <c r="A204" s="11" t="inlineStr">
@@ -11516,11 +11715,15 @@
       </c>
       <c r="H204" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="I204" s="11" t="n"/>
-      <c r="J204" s="12" t="n"/>
+      <c r="J204" s="12" t="inlineStr">
+        <is>
+          <t>Pendiente (por indicación, para otro momento). El middleware de suscripción global (SuscripcionVigenteHandler, HU-160) ya aplica a estos endpoints cuando se construyan.</t>
+        </is>
+      </c>
     </row>
     <row r="205" ht="41.4" customHeight="1" s="19">
       <c r="A205" s="11" t="inlineStr">
@@ -11558,11 +11761,15 @@
       </c>
       <c r="H205" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="I205" s="11" t="n"/>
-      <c r="J205" s="12" t="n"/>
+      <c r="J205" s="12" t="inlineStr">
+        <is>
+          <t>Pendiente (por indicación, para otro momento). El middleware de suscripción global (SuscripcionVigenteHandler, HU-160) ya aplica a estos endpoints cuando se construyan.</t>
+        </is>
+      </c>
     </row>
     <row r="206" ht="27.6" customHeight="1" s="19">
       <c r="A206" s="11" t="inlineStr">
@@ -11726,11 +11933,15 @@
       </c>
       <c r="H209" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I209" s="11" t="n"/>
-      <c r="J209" s="12" t="n"/>
+      <c r="J209" s="12" t="inlineStr">
+        <is>
+          <t>Seguridad a nivel de datos: SEL/UPS acotan por cliente + usuario + planta (Cliente_Instalacion_Usuario); un usuario no ve ni escribe ejecuciones de una planta a la que no pertenece. Verificado: usuario sin planta obtiene 0 filas.</t>
+        </is>
+      </c>
     </row>
     <row r="210" ht="27.6" customHeight="1" s="19">
       <c r="A210" s="11" t="inlineStr">
@@ -13616,11 +13827,15 @@
       </c>
       <c r="H254" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I254" s="11" t="n"/>
-      <c r="J254" s="12" t="n"/>
+      <c r="J254" s="12" t="inlineStr">
+        <is>
+          <t>Modelo alineado (BD/205): se quitó UX_TCA_GLOBAL_CODIGO (código único global, que contradecía el criterio) y quedó UX_TCA_CLIENTE_CODIGO (único por cliente). Tabla estaba vacía.</t>
+        </is>
+      </c>
     </row>
     <row r="255" ht="41.4" customHeight="1" s="19">
       <c r="A255" s="11" t="inlineStr">
@@ -13658,11 +13873,15 @@
       </c>
       <c r="H255" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I255" s="11" t="n"/>
-      <c r="J255" s="12" t="n"/>
+      <c r="J255" s="12" t="inlineStr">
+        <is>
+          <t>BD/205: SEL_TAREA_CATEGORIA reescrito (el anterior estaba roto: columnas TCA_USUARIO_ACT/TCA_FECHA_ACT inexistentes, sin filtro por cliente, sin escapar). Un solo SP para grilla y ficha; filtros @ID/@CLIENTE/@FILTRO/@HABILITADO; @FILTRO escapado; ORDER BY estable (orden, código).</t>
+        </is>
+      </c>
     </row>
     <row r="256" ht="41.4" customHeight="1" s="19">
       <c r="A256" s="11" t="inlineStr">
@@ -13700,11 +13919,15 @@
       </c>
       <c r="H256" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I256" s="11" t="n"/>
-      <c r="J256" s="12" t="n"/>
+      <c r="J256" s="12" t="inlineStr">
+        <is>
+          <t>BD/205: INS_TAREA_CATEGORIA en transacción, valida código único por cliente, sella con FNC_PAIS_HORA. Verificado: rechaza código duplicado (msg 2) y normaliza a mayúsculas.</t>
+        </is>
+      </c>
     </row>
     <row r="257" ht="41.4" customHeight="1" s="19">
       <c r="A257" s="11" t="inlineStr">
@@ -13742,11 +13965,15 @@
       </c>
       <c r="H257" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I257" s="11" t="n"/>
-      <c r="J257" s="12" t="n"/>
+      <c r="J257" s="12" t="inlineStr">
+        <is>
+          <t>BD/205: UPD_TAREA_CATEGORIA con ISNULL(@X, columna) (lo que la ficha no manda se conserva) y código único por cliente excluyendo el propio. Verificado.</t>
+        </is>
+      </c>
     </row>
     <row r="258" ht="41.4" customHeight="1" s="19">
       <c r="A258" s="11" t="inlineStr">
@@ -13784,11 +14011,15 @@
       </c>
       <c r="H258" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I258" s="11" t="n"/>
-      <c r="J258" s="12" t="n"/>
+      <c r="J258" s="12" t="inlineStr">
+        <is>
+          <t>BD/205: DEL_TAREA_CATEGORIA baja lógica (tca_habilitado=0); rechaza si la categoría tiene tareas asociadas (tar_tarea_categoria) en vez de dejarlas huérfanas. Verificado.</t>
+        </is>
+      </c>
     </row>
     <row r="259" ht="41.4" customHeight="1" s="19">
       <c r="A259" s="11" t="inlineStr">
@@ -13826,11 +14057,15 @@
       </c>
       <c r="H259" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I259" s="11" t="n"/>
-      <c r="J259" s="12" t="n"/>
+      <c r="J259" s="12" t="inlineStr">
+        <is>
+          <t>BD/205: datos de prueba (PREVENTIVO/CORRECTIVO/INSPECCION del cliente 1, con color y orden; idempotentes por código).</t>
+        </is>
+      </c>
     </row>
     <row r="260" ht="41.4" customHeight="1" s="19">
       <c r="A260" s="11" t="inlineStr">
@@ -13868,11 +14103,15 @@
       </c>
       <c r="H260" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I260" s="11" t="n"/>
-      <c r="J260" s="12" t="n"/>
+      <c r="J260" s="12" t="inlineStr">
+        <is>
+          <t>Web TareaCategorias.aspx: grilla con búsqueda, filtro de habilitados y botón Nuevo; muestra el color como muestra. Compila exitcode 0.</t>
+        </is>
+      </c>
     </row>
     <row r="261" ht="27.6" customHeight="1" s="19">
       <c r="A261" s="11" t="inlineStr">
@@ -13910,11 +14149,15 @@
       </c>
       <c r="H261" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I261" s="11" t="n"/>
-      <c r="J261" s="12" t="n"/>
+      <c r="J261" s="12" t="inlineStr">
+        <is>
+          <t>Web TareaCategoria.aspx en RadWindow (SigmaModal) con clases sigma-modal-*: código/nombre/color/orden/habilitado, validadores y Guardar/Cerrar.</t>
+        </is>
+      </c>
     </row>
     <row r="262" ht="41.4" customHeight="1" s="19">
       <c r="A262" s="11" t="inlineStr">
@@ -13952,11 +14195,15 @@
       </c>
       <c r="H262" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I262" s="11" t="n"/>
-      <c r="J262" s="12" t="n"/>
+      <c r="J262" s="12" t="inlineStr">
+        <is>
+          <t>BD/206: registra listado (visible) y ficha (oculta) en Menus con permiso VER TAREAS; sin fila en Menus la pantalla no se abre.</t>
+        </is>
+      </c>
     </row>
     <row r="263" ht="55.2" customHeight="1" s="19">
       <c r="A263" s="11" t="inlineStr">
@@ -13994,11 +14241,15 @@
       </c>
       <c r="H263" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t>Terminada</t>
         </is>
       </c>
       <c r="I263" s="11" t="n"/>
-      <c r="J263" s="12" t="n"/>
+      <c r="J263" s="12" t="inlineStr">
+        <is>
+          <t>Seguridad server-side: Token.Puede('CREAR EDITAR TAREAS') revalidado en btnGuardar_Click (no se esconde el botón); función Crear y editar en Menu_Funcion; SEL/listado filtran por cliente en sesión.</t>
+        </is>
+      </c>
     </row>
     <row r="264" ht="41.4" customHeight="1" s="19">
       <c r="A264" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Sprint 4: las 31 tareas pendientes del plan de mantenimiento pasan a Bryan
Bryan continua el epico del plan -HU-080 a HU-087-, asi que sus pendientes se
reasignan a un solo dueño: 21 venian de Catalina, 7 de Emilio y 3 ya eran de
Bryan.

Esas 3 estaban BLOQUEADAS y dejan de estarlo: eran las pruebas de HU-082, que
esperaban la pantalla de actividades: ahora el desarrollo y su verificacion
tienen el mismo responsable, asi que no hay a quien esperar.

Cada fila anota en Observaciones de donde vino, para que el reparto sea
auditable en la retro.

El backup previo queda en SIGMA_Sprint_Backlog_S4_BACKUP_PRE_REASIGNACION_PLAN.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S4.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S4.xlsx
@@ -3735,7 +3735,7 @@
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -3744,7 +3744,11 @@
         </is>
       </c>
       <c r="I16" s="11" t="n"/>
-      <c r="J16" s="12" t="n"/>
+      <c r="J16" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="41.45" customHeight="1" s="19">
       <c r="A17" s="11" t="inlineStr">
@@ -3777,7 +3781,7 @@
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
@@ -3786,7 +3790,11 @@
         </is>
       </c>
       <c r="I17" s="11" t="n"/>
-      <c r="J17" s="12" t="n"/>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="27.6" customHeight="1" s="19">
       <c r="A18" s="11" t="inlineStr">
@@ -3819,7 +3827,7 @@
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -3828,7 +3836,11 @@
         </is>
       </c>
       <c r="I18" s="11" t="n"/>
-      <c r="J18" s="12" t="n"/>
+      <c r="J18" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="55.15" customHeight="1" s="19">
       <c r="A19" s="11" t="inlineStr">
@@ -4317,7 +4329,7 @@
       </c>
       <c r="G29" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H29" s="11" t="inlineStr">
@@ -4326,7 +4338,11 @@
         </is>
       </c>
       <c r="I29" s="11" t="n"/>
-      <c r="J29" s="12" t="n"/>
+      <c r="J29" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="41.45" customHeight="1" s="19">
       <c r="A30" s="11" t="inlineStr">
@@ -4359,7 +4375,7 @@
       </c>
       <c r="G30" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -4368,7 +4384,11 @@
         </is>
       </c>
       <c r="I30" s="11" t="n"/>
-      <c r="J30" s="12" t="n"/>
+      <c r="J30" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="27.6" customHeight="1" s="19">
       <c r="A31" s="11" t="inlineStr">
@@ -4401,7 +4421,7 @@
       </c>
       <c r="G31" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H31" s="11" t="inlineStr">
@@ -4410,7 +4430,11 @@
         </is>
       </c>
       <c r="I31" s="11" t="n"/>
-      <c r="J31" s="12" t="n"/>
+      <c r="J31" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="27.6" customHeight="1" s="19">
       <c r="A32" s="11" t="inlineStr">
@@ -5109,7 +5133,7 @@
       </c>
       <c r="G46" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -5118,7 +5142,11 @@
         </is>
       </c>
       <c r="I46" s="11" t="n"/>
-      <c r="J46" s="12" t="n"/>
+      <c r="J46" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="41.45" customHeight="1" s="19">
       <c r="A47" s="11" t="inlineStr">
@@ -5151,7 +5179,7 @@
       </c>
       <c r="G47" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H47" s="11" t="inlineStr">
@@ -5160,7 +5188,11 @@
         </is>
       </c>
       <c r="I47" s="11" t="n"/>
-      <c r="J47" s="12" t="n"/>
+      <c r="J47" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="27.6" customHeight="1" s="19">
       <c r="A48" s="11" t="inlineStr">
@@ -5193,7 +5225,7 @@
       </c>
       <c r="G48" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -5202,7 +5234,11 @@
         </is>
       </c>
       <c r="I48" s="11" t="n"/>
-      <c r="J48" s="12" t="n"/>
+      <c r="J48" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="27.6" customHeight="1" s="19">
       <c r="A49" s="11" t="inlineStr">
@@ -5235,7 +5271,7 @@
       </c>
       <c r="G49" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H49" s="11" t="inlineStr">
@@ -5244,7 +5280,11 @@
         </is>
       </c>
       <c r="I49" s="11" t="n"/>
-      <c r="J49" s="12" t="n"/>
+      <c r="J49" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="27.6" customHeight="1" s="19">
       <c r="A50" s="11" t="inlineStr">
@@ -5277,7 +5317,7 @@
       </c>
       <c r="G50" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
@@ -5286,7 +5326,11 @@
         </is>
       </c>
       <c r="I50" s="11" t="n"/>
-      <c r="J50" s="12" t="n"/>
+      <c r="J50" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="55.15" customHeight="1" s="19">
       <c r="A51" s="11" t="inlineStr">
@@ -5319,7 +5363,7 @@
       </c>
       <c r="G51" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H51" s="11" t="inlineStr">
@@ -5328,7 +5372,11 @@
         </is>
       </c>
       <c r="I51" s="11" t="n"/>
-      <c r="J51" s="12" t="n"/>
+      <c r="J51" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="41.45" customHeight="1" s="19">
       <c r="A52" s="11" t="inlineStr">
@@ -5361,7 +5409,7 @@
       </c>
       <c r="G52" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
@@ -5370,7 +5418,11 @@
         </is>
       </c>
       <c r="I52" s="11" t="n"/>
-      <c r="J52" s="12" t="n"/>
+      <c r="J52" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="41.45" customHeight="1" s="19">
       <c r="A53" s="11" t="inlineStr">
@@ -5403,7 +5455,7 @@
       </c>
       <c r="G53" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H53" s="11" t="inlineStr">
@@ -5412,7 +5464,11 @@
         </is>
       </c>
       <c r="I53" s="11" t="n"/>
-      <c r="J53" s="12" t="n"/>
+      <c r="J53" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="27.6" customHeight="1" s="19">
       <c r="A54" s="11" t="inlineStr">
@@ -5445,7 +5501,7 @@
       </c>
       <c r="G54" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
@@ -5454,7 +5510,11 @@
         </is>
       </c>
       <c r="I54" s="11" t="n"/>
-      <c r="J54" s="12" t="n"/>
+      <c r="J54" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="41.45" customHeight="1" s="19">
       <c r="A55" s="11" t="inlineStr">
@@ -5487,7 +5547,7 @@
       </c>
       <c r="G55" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H55" s="11" t="inlineStr">
@@ -5496,7 +5556,11 @@
         </is>
       </c>
       <c r="I55" s="11" t="n"/>
-      <c r="J55" s="12" t="n"/>
+      <c r="J55" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="41.45" customHeight="1" s="19">
       <c r="A56" s="11" t="inlineStr">
@@ -5534,13 +5598,13 @@
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Por hacer</t>
         </is>
       </c>
       <c r="I56" s="11" t="n"/>
       <c r="J56" s="12" t="inlineStr">
         <is>
-          <t>HU-082 (actividades) es de Catalina y no está en el repo: sin actividades no hay casos que ejecutar.</t>
+          <t>HU-082 (actividades) es de Catalina y no está en el repo: sin actividades no hay casos que ejecutar.  Desbloqueada (24-09-2026): el desarrollo del que dependía pasa al mismo responsable.</t>
         </is>
       </c>
     </row>
@@ -5580,13 +5644,13 @@
       </c>
       <c r="H57" s="11" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Por hacer</t>
         </is>
       </c>
       <c r="I57" s="11" t="n"/>
       <c r="J57" s="12" t="inlineStr">
         <is>
-          <t>Espera HU-082.</t>
+          <t>Espera HU-082.  Desbloqueada (24-09-2026): el desarrollo del que dependía pasa al mismo responsable.</t>
         </is>
       </c>
     </row>
@@ -5626,13 +5690,13 @@
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>Bloqueada</t>
+          <t>Por hacer</t>
         </is>
       </c>
       <c r="I58" s="11" t="n"/>
       <c r="J58" s="12" t="inlineStr">
         <is>
-          <t>Espera HU-082 y a la PO.</t>
+          <t>Espera HU-082 y a la PO.  Desbloqueada (24-09-2026): el desarrollo del que dependía pasa al mismo responsable.</t>
         </is>
       </c>
     </row>
@@ -7061,7 +7125,7 @@
       </c>
       <c r="G90" s="12" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H90" s="11" t="inlineStr">
@@ -7070,7 +7134,11 @@
         </is>
       </c>
       <c r="I90" s="11" t="n"/>
-      <c r="J90" s="12" t="n"/>
+      <c r="J90" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="27.6" customHeight="1" s="19">
       <c r="A91" s="11" t="inlineStr">
@@ -7103,7 +7171,7 @@
       </c>
       <c r="G91" s="12" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H91" s="11" t="inlineStr">
@@ -7112,7 +7180,11 @@
         </is>
       </c>
       <c r="I91" s="11" t="n"/>
-      <c r="J91" s="12" t="n"/>
+      <c r="J91" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="27.6" customHeight="1" s="19">
       <c r="A92" s="11" t="inlineStr">
@@ -9689,7 +9761,7 @@
       </c>
       <c r="G148" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H148" s="11" t="inlineStr">
@@ -9698,7 +9770,11 @@
         </is>
       </c>
       <c r="I148" s="11" t="n"/>
-      <c r="J148" s="12" t="n"/>
+      <c r="J148" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="41.45" customHeight="1" s="19">
       <c r="A149" s="11" t="inlineStr">
@@ -9731,7 +9807,7 @@
       </c>
       <c r="G149" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H149" s="11" t="inlineStr">
@@ -9740,7 +9816,11 @@
         </is>
       </c>
       <c r="I149" s="11" t="n"/>
-      <c r="J149" s="12" t="n"/>
+      <c r="J149" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="41.45" customHeight="1" s="19">
       <c r="A150" s="11" t="inlineStr">
@@ -9773,7 +9853,7 @@
       </c>
       <c r="G150" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H150" s="11" t="inlineStr">
@@ -9782,7 +9862,11 @@
         </is>
       </c>
       <c r="I150" s="11" t="n"/>
-      <c r="J150" s="12" t="n"/>
+      <c r="J150" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="27.6" customHeight="1" s="19">
       <c r="A151" s="11" t="inlineStr">
@@ -9815,7 +9899,7 @@
       </c>
       <c r="G151" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H151" s="11" t="inlineStr">
@@ -9824,7 +9908,11 @@
         </is>
       </c>
       <c r="I151" s="11" t="n"/>
-      <c r="J151" s="12" t="n"/>
+      <c r="J151" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="27.6" customHeight="1" s="19">
       <c r="A152" s="11" t="inlineStr">
@@ -9857,7 +9945,7 @@
       </c>
       <c r="G152" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H152" s="11" t="inlineStr">
@@ -9866,7 +9954,11 @@
         </is>
       </c>
       <c r="I152" s="11" t="n"/>
-      <c r="J152" s="12" t="n"/>
+      <c r="J152" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="153" ht="27.6" customHeight="1" s="19">
       <c r="A153" s="11" t="inlineStr">
@@ -9899,7 +9991,7 @@
       </c>
       <c r="G153" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H153" s="11" t="inlineStr">
@@ -9908,7 +10000,11 @@
         </is>
       </c>
       <c r="I153" s="11" t="n"/>
-      <c r="J153" s="12" t="n"/>
+      <c r="J153" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="154" ht="55.15" customHeight="1" s="19">
       <c r="A154" s="11" t="inlineStr">
@@ -9941,7 +10037,7 @@
       </c>
       <c r="G154" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H154" s="11" t="inlineStr">
@@ -9950,7 +10046,11 @@
         </is>
       </c>
       <c r="I154" s="11" t="n"/>
-      <c r="J154" s="12" t="n"/>
+      <c r="J154" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="41.45" customHeight="1" s="19">
       <c r="A155" s="11" t="inlineStr">
@@ -9983,7 +10083,7 @@
       </c>
       <c r="G155" s="12" t="inlineStr">
         <is>
-          <t>Catalina Pescio</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H155" s="11" t="inlineStr">
@@ -9992,7 +10092,11 @@
         </is>
       </c>
       <c r="I155" s="11" t="n"/>
-      <c r="J155" s="12" t="n"/>
+      <c r="J155" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="156" ht="41.45" customHeight="1" s="19">
       <c r="A156" s="11" t="inlineStr">
@@ -11259,7 +11363,7 @@
       </c>
       <c r="G183" s="12" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H183" s="11" t="inlineStr">
@@ -11268,7 +11372,11 @@
         </is>
       </c>
       <c r="I183" s="11" t="n"/>
-      <c r="J183" s="12" t="n"/>
+      <c r="J183" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="184" ht="41.45" customHeight="1" s="19">
       <c r="A184" s="11" t="inlineStr">
@@ -11301,7 +11409,7 @@
       </c>
       <c r="G184" s="12" t="inlineStr">
         <is>
-          <t>Emilio Fuentes</t>
+          <t>Bryan Chávez</t>
         </is>
       </c>
       <c r="H184" s="11" t="inlineStr">
@@ -11310,7 +11418,11 @@
         </is>
       </c>
       <c r="I184" s="11" t="n"/>
-      <c r="J184" s="12" t="n"/>
+      <c r="J184" s="12" t="inlineStr">
+        <is>
+          <t>Reasignada a Bryan Chávez (24-09-2026): continúa el épico del plan de mantenimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="185" ht="27.6" customHeight="1" s="19">
       <c r="A185" s="11" t="inlineStr">

</xml_diff>

<commit_message>
HU-104: pruebas de Comentar una tarea y cierre
Cierra HU-104 (Comentar una tarea). El desarrollo (comentarios por ocurrencia
en el centro, API y seguridad) ya estaba integrado por Bryan.

Pruebas ejecutadas en vivo (Selenium + verificación en BD) sobre TAR-001:
- CA-1: un comentario queda con el nombre del autor y la fecha (Catalina Pescio
  · Web · 24 sept 2026) y no puede editarse ni eliminarse (el hilo solo ofrece
  "Responder"; "se conservan como registro").
- CA-2: la respuesta se muestra anidada bajo el comentario original
  (tco_comentario_padre = 7 en BD).

Documentación: el endpoint POST /api/tareas/{id}/comentarios ya está documentado
con comentarios XML de Swagger en API/Controllers/TareasController.cs; decisiones
del módulo en MD/SIGMA_MODULO_TAREAS.md. Informe con capturas en
Fase 2/Pruebas/SIGMA_Pruebas_HU-104.docx.

S4: T-4334 y T-4335 -> Terminada; historia HU-104 -> Terminada.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S4.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S4.xlsx
@@ -3076,7 +3076,7 @@
       </c>
       <c r="N29" s="13" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="O29" s="14" t="inlineStr">
@@ -3086,7 +3086,7 @@
       </c>
       <c r="P29" s="14" t="inlineStr">
         <is>
-          <t>Hecho y verificado el 12-09-2026; pendiente validación de la PO.</t>
+          <t xml:space="preserve">Hecho y verificado por Bryan (12-09-2026). Pruebas (CA-1 comentario con nombre/fecha e inmutable; CA-2 respuesta anidada) y documentación (endpoint API en Swagger + MD) cerradas por Catalina (24-09-2026). Pendiente solo validación de la PO.</t>
         </is>
       </c>
     </row>
@@ -15558,11 +15558,15 @@
       </c>
       <c r="H278" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="I278" s="11" t="n"/>
-      <c r="J278" s="12" t="n"/>
+      <c r="J278" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cerrada por Catalina Pescio (24-09-2026).</t>
+        </is>
+      </c>
     </row>
     <row r="279" ht="41.45" customHeight="1" s="19">
       <c r="A279" s="11" t="inlineStr">
@@ -15600,11 +15604,15 @@
       </c>
       <c r="H279" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="I279" s="11" t="n"/>
-      <c r="J279" s="12" t="n"/>
+      <c r="J279" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cerrada por Catalina Pescio (24-09-2026).</t>
+        </is>
+      </c>
     </row>
     <row r="280" ht="27.6" customHeight="1" s="19"/>
     <row r="281" ht="27.6" customHeight="1" s="19"/>

</xml_diff>

<commit_message>
HU-092: mantenedor de dependencias entre ítems + cierre
Construye el mantenedor web para definir dependencias entre ítems de una
pauta (un ítem se muestra/oculta/requiere/bloquea según cómo se respondió
otro ítem, con operador y valor):

- BD/309: SP SEL/INS/UPD/DEL_CHECKLIST_ITEM_DEPENDENCIA. El alta valida
  misma pauta, no auto-dependencia (CA-2) y no dependencia inversa (ciclo).
- Web: ChecklistItemDependencias.aspx (listado) + ChecklistItemDependencia.aspx
  (ficha) + controlador y modelo. El combo de ítems reutiliza
  SEL_CHECKLIST_ITEM_LISTA (HU-091).
- BD/310: permisos VER/CREAR EDITAR DEPENDENCIAS + menú bajo Centro de
  Mantenimiento.
- Pruebas (Selenium) y evidencia BD: alta OK y rechazo de dependencia
  circular. Informe Fase 2/Pruebas/SIGMA_Pruebas_HU-092.docx, sección en
  MD/SIGMA_MODULO_TAREAS.md y cierre en el backlog S4.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S4.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S4.xlsx
@@ -2705,7 +2705,7 @@
       </c>
       <c r="N24" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="O24" s="12" t="inlineStr">
@@ -2713,7 +2713,11 @@
           <t>Catalina Pescio</t>
         </is>
       </c>
-      <c r="P24" s="12" t="n"/>
+      <c r="P24" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mantenedor de dependencias entre ítems construido: BD SP SEL/INS/UPD/DEL (BD/309), Web listado+ficha+controlador+modelo y menú/permisos (BD/310). Pruebas y documentación cerradas por Catalina Pescio (29-09-2026).</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="55.15" customHeight="1" s="19">
       <c r="A25" s="13" t="inlineStr">
@@ -12822,11 +12826,15 @@
       </c>
       <c r="H212" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="I212" s="11" t="n"/>
-      <c r="J212" s="12" t="n"/>
+      <c r="J212" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada por Catalina Pescio — 29-09-2026.</t>
+        </is>
+      </c>
     </row>
     <row r="213" ht="27.6" customHeight="1" s="19">
       <c r="A213" s="11" t="inlineStr">
@@ -12864,11 +12872,15 @@
       </c>
       <c r="H213" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="I213" s="11" t="n"/>
-      <c r="J213" s="12" t="n"/>
+      <c r="J213" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada por Catalina Pescio — 29-09-2026.</t>
+        </is>
+      </c>
     </row>
     <row r="214" ht="55.15" customHeight="1" s="19">
       <c r="A214" s="11" t="inlineStr">
@@ -12906,11 +12918,15 @@
       </c>
       <c r="H214" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="I214" s="11" t="n"/>
-      <c r="J214" s="12" t="n"/>
+      <c r="J214" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada por Catalina Pescio — 29-09-2026.</t>
+        </is>
+      </c>
     </row>
     <row r="215" ht="41.45" customHeight="1" s="19">
       <c r="A215" s="11" t="inlineStr">
@@ -12948,11 +12964,15 @@
       </c>
       <c r="H215" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="I215" s="11" t="n"/>
-      <c r="J215" s="12" t="n"/>
+      <c r="J215" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada por Catalina Pescio — 29-09-2026.</t>
+        </is>
+      </c>
     </row>
     <row r="216" ht="41.45" customHeight="1" s="19">
       <c r="A216" s="11" t="inlineStr">
@@ -12990,11 +13010,15 @@
       </c>
       <c r="H216" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="I216" s="11" t="n"/>
-      <c r="J216" s="12" t="n"/>
+      <c r="J216" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada por Catalina Pescio — 29-09-2026.</t>
+        </is>
+      </c>
     </row>
     <row r="217" ht="41.45" customHeight="1" s="19">
       <c r="A217" s="11" t="inlineStr">
@@ -13032,11 +13056,15 @@
       </c>
       <c r="H217" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="I217" s="11" t="n"/>
-      <c r="J217" s="12" t="n"/>
+      <c r="J217" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada por Catalina Pescio — 29-09-2026.</t>
+        </is>
+      </c>
     </row>
     <row r="218" ht="41.45" customHeight="1" s="19">
       <c r="A218" s="11" t="inlineStr">
@@ -13074,11 +13102,15 @@
       </c>
       <c r="H218" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="I218" s="11" t="n"/>
-      <c r="J218" s="12" t="n"/>
+      <c r="J218" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada por Catalina Pescio — 29-09-2026.</t>
+        </is>
+      </c>
     </row>
     <row r="219" ht="27.6" customHeight="1" s="19">
       <c r="A219" s="11" t="inlineStr">
@@ -13116,11 +13148,15 @@
       </c>
       <c r="H219" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="I219" s="11" t="n"/>
-      <c r="J219" s="12" t="n"/>
+      <c r="J219" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada por Catalina Pescio — 29-09-2026.</t>
+        </is>
+      </c>
     </row>
     <row r="220" ht="27.6" customHeight="1" s="19">
       <c r="A220" s="11" t="inlineStr">
@@ -13158,11 +13194,15 @@
       </c>
       <c r="H220" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="I220" s="11" t="n"/>
-      <c r="J220" s="12" t="n"/>
+      <c r="J220" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada por Catalina Pescio — 29-09-2026.</t>
+        </is>
+      </c>
     </row>
     <row r="221" ht="27.6" customHeight="1" s="19">
       <c r="A221" s="11" t="inlineStr">
@@ -13200,11 +13240,15 @@
       </c>
       <c r="H221" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="I221" s="11" t="n"/>
-      <c r="J221" s="12" t="n"/>
+      <c r="J221" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terminada por Catalina Pescio — 29-09-2026.</t>
+        </is>
+      </c>
     </row>
     <row r="222" ht="27.6" customHeight="1" s="19">
       <c r="A222" s="11" t="inlineStr">
@@ -13242,11 +13286,15 @@
       </c>
       <c r="H222" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="I222" s="11" t="n"/>
-      <c r="J222" s="12" t="n"/>
+      <c r="J222" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cerrada por Catalina Pescio (pruebas y documentación del módulo) — 29-09-2026.</t>
+        </is>
+      </c>
     </row>
     <row r="223" ht="27.6" customHeight="1" s="19">
       <c r="A223" s="11" t="inlineStr">
@@ -13284,11 +13332,15 @@
       </c>
       <c r="H223" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
+          <t xml:space="preserve">Terminada</t>
         </is>
       </c>
       <c r="I223" s="11" t="n"/>
-      <c r="J223" s="12" t="n"/>
+      <c r="J223" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cerrada por Catalina Pescio (pruebas y documentación del módulo) — 29-09-2026.</t>
+        </is>
+      </c>
     </row>
     <row r="224" ht="55.15" customHeight="1" s="19">
       <c r="A224" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Sprint Backlog S4: HU-091 y HU-097 con criterios verificados y horas reales
Los 6 criterios pasan a Verificado = Sí (casos en el informe de pruebas del
Sprint 4), se quita de HU-091 la nota de validación pendiente (T-4137 ya
conforme) y las 20 tareas sin horas reales toman las estimadas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S4.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S4.xlsx
@@ -1965,7 +1965,7 @@
       </c>
       <c r="P14" s="12" t="inlineStr">
         <is>
-          <t>Mantenedor de umbrales/acciones construido por Catalina: SP SEL/INS/UPD/DEL_CHECKLIST_ITEM_VALIDACION (BD/307), pantallas ChecklistItemValidacion(s) + controller/modelo, permisos/menú (BD/308). Pruebas (CA-1: 84-&gt;crítica; CA-2/3/4 definición+runtime) y documentación cerradas (29-09-2026). Pendiente solo la validación funcional con la PO (T-4137).</t>
+          <t>Mantenedor de umbrales/acciones construido por Catalina: SP SEL/INS/UPD/DEL_CHECKLIST_ITEM_VALIDACION (BD/307), pantallas ChecklistItemValidacion(s) + controller/modelo, permisos/menú (BD/308). Pruebas (CA-1: 84-&gt;crítica; CA-2/3/4 definición+runtime) y documentación cerradas (29-09-2026). Validación funcional con la PO conforme (T-4137).</t>
         </is>
       </c>
     </row>
@@ -7719,7 +7719,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I101" s="11" t="n"/>
+      <c r="I101" s="11" t="n">
+        <v>0.75</v>
+      </c>
       <c r="J101" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -7765,7 +7767,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I102" s="11" t="n"/>
+      <c r="I102" s="11" t="n">
+        <v>0.75</v>
+      </c>
       <c r="J102" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -7811,7 +7815,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I103" s="11" t="n"/>
+      <c r="I103" s="11" t="n">
+        <v>0.75</v>
+      </c>
       <c r="J103" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -7857,7 +7863,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I104" s="11" t="n"/>
+      <c r="I104" s="11" t="n">
+        <v>0.5</v>
+      </c>
       <c r="J104" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -7903,7 +7911,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I105" s="11" t="n"/>
+      <c r="I105" s="11" t="n">
+        <v>0.5</v>
+      </c>
       <c r="J105" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -7949,7 +7959,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I106" s="11" t="n"/>
+      <c r="I106" s="11" t="n">
+        <v>0.5</v>
+      </c>
       <c r="J106" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -7995,7 +8007,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I107" s="11" t="n"/>
+      <c r="I107" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="J107" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -8041,7 +8055,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I108" s="11" t="n"/>
+      <c r="I108" s="11" t="n">
+        <v>0.75</v>
+      </c>
       <c r="J108" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -8087,7 +8103,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I109" s="11" t="n"/>
+      <c r="I109" s="11" t="n">
+        <v>0.75</v>
+      </c>
       <c r="J109" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -8133,7 +8151,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I110" s="11" t="n"/>
+      <c r="I110" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="J110" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -8179,7 +8199,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I111" s="11" t="n"/>
+      <c r="I111" s="11" t="n">
+        <v>1.25</v>
+      </c>
       <c r="J111" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -8225,7 +8247,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I112" s="11" t="n"/>
+      <c r="I112" s="11" t="n">
+        <v>0.5</v>
+      </c>
       <c r="J112" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -14439,7 +14463,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I246" s="11" t="n"/>
+      <c r="I246" s="11" t="n">
+        <v>0.75</v>
+      </c>
       <c r="J246" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -14485,7 +14511,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I247" s="11" t="n"/>
+      <c r="I247" s="11" t="n">
+        <v>0.75</v>
+      </c>
       <c r="J247" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -14531,7 +14559,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I248" s="11" t="n"/>
+      <c r="I248" s="11" t="n">
+        <v>0.5</v>
+      </c>
       <c r="J248" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -14577,7 +14607,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I249" s="11" t="n"/>
+      <c r="I249" s="11" t="n">
+        <v>0.5</v>
+      </c>
       <c r="J249" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -14623,7 +14655,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I250" s="11" t="n"/>
+      <c r="I250" s="11" t="n">
+        <v>1.5</v>
+      </c>
       <c r="J250" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -14669,7 +14703,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I251" s="11" t="n"/>
+      <c r="I251" s="11" t="n">
+        <v>0.5</v>
+      </c>
       <c r="J251" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -14715,7 +14751,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I252" s="11" t="n"/>
+      <c r="I252" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="J252" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -14761,7 +14799,9 @@
           <t>Terminada</t>
         </is>
       </c>
-      <c r="I253" s="11" t="n"/>
+      <c r="I253" s="11" t="n">
+        <v>0.25</v>
+      </c>
       <c r="J253" s="12" t="inlineStr">
         <is>
           <t>Cerrada por Catalina Pescio (29-09-2026).</t>
@@ -17110,7 +17150,7 @@
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -17142,7 +17182,7 @@
       </c>
       <c r="F37" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -17174,7 +17214,7 @@
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -17207,7 +17247,7 @@
       </c>
       <c r="F39" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -18348,7 +18388,7 @@
       </c>
       <c r="F75" s="13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -18380,7 +18420,7 @@
       </c>
       <c r="F76" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -18760,7 +18800,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="19">
       <c r="A16" s="20" t="inlineStr">
         <is>

</xml_diff>